<commit_message>
Program Coding Pahse Defects Checklist
</commit_message>
<xml_diff>
--- a/Docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/Docs/Lab01/Lab01_ReviewReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VVSS\Docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48AA400D-ADFF-4258-A3AA-F9D6DBCF96C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54708136-BCDC-4DA9-8170-65B7BBD871AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="528" yWindow="1476" windowWidth="17280" windowHeight="8880" tabRatio="650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="88">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -190,15 +190,6 @@
     <t>A03</t>
   </si>
   <si>
-    <t>A04</t>
-  </si>
-  <si>
-    <t>A05</t>
-  </si>
-  <si>
-    <t>A08</t>
-  </si>
-  <si>
     <t>A09</t>
   </si>
   <si>
@@ -208,21 +199,12 @@
     <t>A01</t>
   </si>
   <si>
-    <t>Controller-ul contine liste de produse, retete, comanda curenta, produsele din comanda, ar trebui ca repo-ul sa tina aceste liste</t>
-  </si>
-  <si>
     <t>Tipul si categoria baututilor sunt de tip enum, dar in cerinta 3 se specifica ca user-ul poate modifica/sterge/adauga tipuri sau categorii de bauturi.</t>
   </si>
   <si>
-    <t>Lipseste gestionarea rolurilor de Admin/User</t>
-  </si>
-  <si>
     <t>DailyRaportService are o relatie numita "repo" spre interfata Repository si nu este clar din arhitectura ce fel de date se extrag pentru raporturi</t>
   </si>
   <si>
-    <t>Nu, datorita DrinkShopController care detine liste de produse, comenzi, etc, incalcand principiul singurei reposnsabiliati</t>
-  </si>
-  <si>
     <t>A10</t>
   </si>
   <si>
@@ -232,7 +214,82 @@
     <t>ProducTest nu ar trebui sa apara in diagrama</t>
   </si>
   <si>
-    <t>Chiar daca avem clase de validare, arhitectura nu include clar o componenta pentru tratarea erorilor, spre exeplu: ErrorHandler</t>
+    <t>C06</t>
+  </si>
+  <si>
+    <t>DrinkShopContoller line169</t>
+  </si>
+  <si>
+    <t>CsvExporter</t>
+  </si>
+  <si>
+    <t>C08</t>
+  </si>
+  <si>
+    <t>C05</t>
+  </si>
+  <si>
+    <t>C09</t>
+  </si>
+  <si>
+    <t>DrinkShopContoller</t>
+  </si>
+  <si>
+    <t>DrinkShopController - onAddProduct</t>
+  </si>
+  <si>
+    <t>DailyReportService</t>
+  </si>
+  <si>
+    <t>StocService</t>
+  </si>
+  <si>
+    <t>OrderService</t>
+  </si>
+  <si>
+    <t>niciun validator nu este folosit!</t>
+  </si>
+  <si>
+    <t>Validatorii nu sunt legati de clase</t>
+  </si>
+  <si>
+    <t>nu avem validari pentru adaugarea unui element</t>
+  </si>
+  <si>
+    <t xml:space="preserve">din O(NxMxP) -&gt; O(P + (NxM)); N - nr de comenzi, M - nr de produse pe comanda, P - nr total de produse
+</t>
+  </si>
+  <si>
+    <t>Eroare afisata doar in consola</t>
+  </si>
+  <si>
+    <t>Utilizatorul nu este informat de crearea csv-ului</t>
+  </si>
+  <si>
+    <t xml:space="preserve">showError nu este folosit in functia onAddProduct() </t>
+  </si>
+  <si>
+    <t>lipsesc validatorii pnetru onAddProduct</t>
+  </si>
+  <si>
+    <t>Numele "repo" este prea vag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metoda neutilizata public void update(Stoc s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comentarii in functia public List&lt;Order&gt; getAllOrders() {
+</t>
+  </si>
+  <si>
+    <t>CsvExporter este izolvat</t>
+  </si>
+  <si>
+    <t>ReceiptGenerator este izolat</t>
+  </si>
+  <si>
+    <t>DrinkShopApp este izolat</t>
   </si>
 </sst>
 </file>
@@ -481,6 +538,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -523,7 +581,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -850,19 +907,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
       <c r="H2" s="3"/>
       <c r="I2" s="18" t="s">
         <v>30</v>
@@ -886,10 +943,10 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="30"/>
       <c r="H4" s="16" t="s">
         <v>21</v>
       </c>
@@ -904,10 +961,10 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="31"/>
+      <c r="E5" s="32"/>
       <c r="H5" s="16" t="s">
         <v>22</v>
       </c>
@@ -919,15 +976,15 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1180,7 +1237,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="6"/>
@@ -1197,19 +1254,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
       <c r="H2" s="3"/>
       <c r="I2" s="18" t="s">
         <v>30</v>
@@ -1222,7 +1279,7 @@
       <c r="H3" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="40" t="s">
+      <c r="I3" s="26" t="s">
         <v>34</v>
       </c>
       <c r="J3" s="16">
@@ -1233,14 +1290,14 @@
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="40" t="s">
+      <c r="I4" s="26" t="s">
         <v>33</v>
       </c>
       <c r="J4" s="3">
@@ -1251,10 +1308,10 @@
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="34"/>
+      <c r="E5" s="35"/>
       <c r="H5" s="16" t="s">
         <v>22</v>
       </c>
@@ -1266,15 +1323,15 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1295,11 +1352,11 @@
         <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1312,85 +1369,85 @@
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
-        <f t="shared" ref="B12:B26" si="0">B11+1</f>
+        <f>B11+1</f>
         <v>3</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
-        <f t="shared" si="0"/>
+        <f>B12+1</f>
         <v>4</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" s="1"/>
+        <v>55</v>
+      </c>
+      <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
-        <f t="shared" si="0"/>
+        <f>B13+1</f>
         <v>5</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="2"/>
+        <v>60</v>
+      </c>
+      <c r="D14" s="1"/>
       <c r="E14" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B15:B22" si="0">B14+1</f>
         <v>6</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D15" s="1"/>
+        <v>53</v>
+      </c>
+      <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="D16" s="1"/>
       <c r="E16" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="D17" s="1"/>
       <c r="E17" s="2" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
@@ -1399,25 +1456,21 @@
         <v>9</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2" t="s">
-        <v>69</v>
-      </c>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="2"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
@@ -1446,48 +1499,12 @@
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B23" s="3">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="2"/>
-    </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B24" s="3">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B25" s="3">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B26" s="3">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C28" s="11" t="s">
+      <c r="C24" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D28" s="12"/>
-      <c r="E28" s="1">
+      <c r="D24" s="12"/>
+      <c r="E24" s="1">
         <v>0.5</v>
       </c>
     </row>
@@ -1517,7 +1534,7 @@
     <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
     <col min="3" max="3" width="16.33203125" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="62.44140625" style="6" customWidth="1"/>
     <col min="6" max="8" width="8.88671875" style="6"/>
     <col min="9" max="9" width="26.6640625" style="6" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="6"/>
@@ -1528,19 +1545,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
       <c r="H2" s="3"/>
       <c r="I2" s="18" t="s">
         <v>30</v>
@@ -1553,7 +1570,7 @@
       <c r="H3" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="40" t="s">
+      <c r="I3" s="26" t="s">
         <v>34</v>
       </c>
       <c r="J3" s="16">
@@ -1564,14 +1581,14 @@
       <c r="C4" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="D4" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="35"/>
+      <c r="E4" s="36"/>
       <c r="H4" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="40" t="s">
+      <c r="I4" s="26" t="s">
         <v>33</v>
       </c>
       <c r="J4" s="3">
@@ -1582,10 +1599,10 @@
       <c r="C5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="36" t="s">
+      <c r="D5" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="37"/>
+      <c r="E5" s="38"/>
       <c r="H5" s="16" t="s">
         <v>22</v>
       </c>
@@ -1597,15 +1614,15 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
@@ -1621,94 +1638,152 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
+      <c r="C12" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="C13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="C15" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C16" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C17" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+      <c r="C18" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1"/>
+      <c r="C19" s="1" t="s">
+        <v>67</v>
+      </c>
       <c r="D19" s="1"/>
-      <c r="E19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
@@ -1814,7 +1889,9 @@
         <v>8</v>
       </c>
       <c r="D32" s="12"/>
-      <c r="E32" s="1"/>
+      <c r="E32" s="1">
+        <v>0.5</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1854,19 +1931,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
       <c r="H2" s="3"/>
       <c r="I2" s="18" t="s">
         <v>30</v>
@@ -1886,8 +1963,8 @@
       <c r="C4" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
       <c r="H4" s="16" t="s">
         <v>21</v>
       </c>
@@ -1898,8 +1975,8 @@
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
       <c r="H5" s="16" t="s">
         <v>22</v>
       </c>
@@ -1911,8 +1988,8 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
       <c r="F6" s="19"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -2142,11 +2219,11 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="38" t="s">
+      <c r="C32" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="39"/>
-      <c r="E32" s="39"/>
+      <c r="D32" s="40"/>
+      <c r="E32" s="40"/>
       <c r="F32" s="17"/>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.3">

</xml_diff>